<commit_message>
Update 12626434.xlsx - 24 August 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ANISH\OneDrive\Documents\GitHub\daily-routine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762DF7D1-2F43-43DF-806E-0063DA6830AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42F59278-3C52-40EB-B6B5-8F051BB6DE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t>Had regular classes and preparing  for DBMS CA2 at night.</t>
+  </si>
+  <si>
+    <t>No regular classes. Studied at home watching movie and relaxed.</t>
   </si>
 </sst>
 </file>
@@ -1452,7 +1455,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
         <v>46256</v>
       </c>
@@ -1495,7 +1498,7 @@
         <v>58</v>
       </c>
       <c r="N14" s="17" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Daily activity log - 22 September 2026
</commit_message>
<xml_diff>
--- a/12626434.xlsx
+++ b/12626434.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ANISH\OneDrive\Documents\GitHub\daily-routine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D130DF-B1C6-44DE-8F67-98273E163DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762DF7D1-2F43-43DF-806E-0063DA6830AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Attended classes and revised the important topics of DBMS at home.</t>
+  </si>
+  <si>
+    <t>Had regular classes and preparing  for DBMS CA2 at night.</t>
   </si>
 </sst>
 </file>
@@ -2875,27 +2878,51 @@
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+    <row r="45" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A45" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B45" s="14">
+        <v>420</v>
+      </c>
+      <c r="C45" s="14">
+        <v>60</v>
+      </c>
+      <c r="D45" s="14">
+        <v>180</v>
+      </c>
+      <c r="E45" s="14">
+        <v>60</v>
+      </c>
+      <c r="F45" s="14">
+        <v>300</v>
+      </c>
+      <c r="G45" s="14">
+        <v>6</v>
+      </c>
+      <c r="H45" s="14">
+        <v>60</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N45" s="17" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" s="13"/>

</xml_diff>